<commit_message>
Brisas, mirador, basa y demas
</commit_message>
<xml_diff>
--- a/2026/BELGRANO 1646/Abril/Abril-BLG1646.xlsx
+++ b/2026/BELGRANO 1646/Abril/Abril-BLG1646.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistemax\Desktop\rc-consorcio2025\2026\BELGRANO 1646\Abril\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82C2FB3-30D3-424D-812D-80D6EB102191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4985B0C-F206-4B9F-8049-4552540BB5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -523,7 +523,7 @@
     <numFmt numFmtId="166" formatCode="_-&quot;$&quot;\ * #,##0_-;\-&quot;$&quot;\ * #,##0_-;_-&quot;$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -685,13 +685,6 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1095,7 +1088,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="209">
+  <cellXfs count="208">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1295,7 +1288,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="6" fontId="23" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="2" fillId="3" borderId="18" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="43" fontId="2" fillId="3" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1383,6 +1375,9 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="44" fontId="0" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1451,9 +1446,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1873,13 +1865,13 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="90"/>
-      <c r="B1" s="155" t="s">
+      <c r="B1" s="154" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="155"/>
-      <c r="D1" s="155"/>
-      <c r="E1" s="155"/>
-      <c r="F1" s="156"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="155"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
@@ -1983,29 +1975,29 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="78"/>
-      <c r="B14" s="159" t="s">
+      <c r="B14" s="158" t="s">
         <v>118</v>
       </c>
-      <c r="C14" s="160"/>
-      <c r="D14" s="161"/>
+      <c r="C14" s="159"/>
+      <c r="D14" s="160"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="78"/>
-      <c r="B15" s="162"/>
-      <c r="C15" s="163"/>
-      <c r="D15" s="164"/>
+      <c r="B15" s="161"/>
+      <c r="C15" s="162"/>
+      <c r="D15" s="163"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="78"/>
-      <c r="B16" s="162"/>
-      <c r="C16" s="163"/>
-      <c r="D16" s="164"/>
+      <c r="B16" s="161"/>
+      <c r="C16" s="162"/>
+      <c r="D16" s="163"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="78"/>
-      <c r="B17" s="165"/>
-      <c r="C17" s="166"/>
-      <c r="D17" s="167"/>
+      <c r="B17" s="164"/>
+      <c r="C17" s="165"/>
+      <c r="D17" s="166"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="78"/>
@@ -2047,7 +2039,7 @@
         <v>122</v>
       </c>
       <c r="C22" s="79"/>
-      <c r="D22" s="154"/>
+      <c r="D22" s="153"/>
       <c r="E22" s="82"/>
       <c r="F22" s="82"/>
     </row>
@@ -2827,11 +2819,11 @@
       </c>
     </row>
     <row r="60" spans="1:10" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="182" t="s">
+      <c r="A60" s="181" t="s">
         <v>136</v>
       </c>
-      <c r="B60" s="183"/>
-      <c r="C60" s="184"/>
+      <c r="B60" s="182"/>
+      <c r="C60" s="183"/>
       <c r="D60" s="37">
         <v>580000</v>
       </c>
@@ -2883,11 +2875,11 @@
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" s="182" t="s">
+      <c r="A62" s="181" t="s">
         <v>129</v>
       </c>
-      <c r="B62" s="183"/>
-      <c r="C62" s="184"/>
+      <c r="B62" s="182"/>
+      <c r="C62" s="183"/>
       <c r="D62" s="37">
         <v>19800</v>
       </c>
@@ -3007,9 +2999,9 @@
       </c>
     </row>
     <row r="66" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="179"/>
-      <c r="B66" s="180"/>
-      <c r="C66" s="181"/>
+      <c r="A66" s="178"/>
+      <c r="B66" s="179"/>
+      <c r="C66" s="180"/>
       <c r="D66" s="37"/>
       <c r="E66" s="60">
         <f t="shared" si="20"/>
@@ -3480,12 +3472,12 @@
       <c r="E96" s="52"/>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A97" s="174" t="s">
+      <c r="A97" s="173" t="s">
         <v>85</v>
       </c>
-      <c r="B97" s="175"/>
-      <c r="C97" s="175"/>
-      <c r="D97" s="175"/>
+      <c r="B97" s="174"/>
+      <c r="C97" s="174"/>
+      <c r="D97" s="174"/>
       <c r="E97" s="73" t="s">
         <v>19</v>
       </c>
@@ -3494,11 +3486,11 @@
       </c>
     </row>
     <row r="98" spans="1:9" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A98" s="171" t="s">
+      <c r="A98" s="170" t="s">
         <v>133</v>
       </c>
-      <c r="B98" s="172"/>
-      <c r="C98" s="173"/>
+      <c r="B98" s="171"/>
+      <c r="C98" s="172"/>
       <c r="D98" s="37">
         <v>512600</v>
       </c>
@@ -3512,11 +3504,11 @@
       </c>
     </row>
     <row r="99" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="176" t="s">
+      <c r="A99" s="175" t="s">
         <v>142</v>
       </c>
-      <c r="B99" s="177"/>
-      <c r="C99" s="178"/>
+      <c r="B99" s="176"/>
+      <c r="C99" s="177"/>
       <c r="D99" s="37">
         <v>300000</v>
       </c>
@@ -3530,11 +3522,11 @@
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A100" s="168" t="s">
+      <c r="A100" s="167" t="s">
         <v>25</v>
       </c>
-      <c r="B100" s="169"/>
-      <c r="C100" s="170"/>
+      <c r="B100" s="168"/>
+      <c r="C100" s="169"/>
       <c r="D100" s="72">
         <f>SUM(D98:D99)</f>
         <v>812600</v>
@@ -3578,8 +3570,8 @@
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D105" s="158"/>
-      <c r="E105" s="158"/>
+      <c r="D105" s="157"/>
+      <c r="E105" s="157"/>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="9" t="s">
@@ -3587,8 +3579,8 @@
       </c>
       <c r="B106" s="10"/>
       <c r="C106" s="11"/>
-      <c r="D106" s="158"/>
-      <c r="E106" s="158"/>
+      <c r="D106" s="157"/>
+      <c r="E106" s="157"/>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="12" t="s">
@@ -3598,8 +3590,8 @@
         <v>10470066.57147561</v>
       </c>
       <c r="C107" s="13"/>
-      <c r="D107" s="158"/>
-      <c r="E107" s="158"/>
+      <c r="D107" s="157"/>
+      <c r="E107" s="157"/>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="14" t="s">
@@ -3612,8 +3604,8 @@
       <c r="C108" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="D108" s="158"/>
-      <c r="E108" s="158"/>
+      <c r="D108" s="157"/>
+      <c r="E108" s="157"/>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="14" t="s">
@@ -3624,8 +3616,8 @@
         <v>-5542413.25</v>
       </c>
       <c r="C109" s="11"/>
-      <c r="D109" s="158"/>
-      <c r="E109" s="158"/>
+      <c r="D109" s="157"/>
+      <c r="E109" s="157"/>
       <c r="G109" s="37"/>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
@@ -3637,8 +3629,8 @@
         <v>-812600</v>
       </c>
       <c r="C110" s="11"/>
-      <c r="D110" s="158"/>
-      <c r="E110" s="158"/>
+      <c r="D110" s="157"/>
+      <c r="E110" s="157"/>
       <c r="G110" s="43"/>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
@@ -3745,34 +3737,34 @@
       <c r="N124" s="6"/>
     </row>
     <row r="127" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B127" s="157"/>
-      <c r="C127" s="157"/>
-      <c r="D127" s="157"/>
-      <c r="E127" s="157"/>
+      <c r="B127" s="156"/>
+      <c r="C127" s="156"/>
+      <c r="D127" s="156"/>
+      <c r="E127" s="156"/>
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B128" s="157"/>
-      <c r="C128" s="157"/>
-      <c r="D128" s="157"/>
-      <c r="E128" s="157"/>
+      <c r="B128" s="156"/>
+      <c r="C128" s="156"/>
+      <c r="D128" s="156"/>
+      <c r="E128" s="156"/>
     </row>
     <row r="129" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B129" s="157"/>
-      <c r="C129" s="157"/>
-      <c r="D129" s="157"/>
-      <c r="E129" s="157"/>
+      <c r="B129" s="156"/>
+      <c r="C129" s="156"/>
+      <c r="D129" s="156"/>
+      <c r="E129" s="156"/>
     </row>
     <row r="130" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B130" s="157"/>
-      <c r="C130" s="157"/>
-      <c r="D130" s="157"/>
-      <c r="E130" s="157"/>
+      <c r="B130" s="156"/>
+      <c r="C130" s="156"/>
+      <c r="D130" s="156"/>
+      <c r="E130" s="156"/>
     </row>
     <row r="131" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B131" s="157"/>
-      <c r="C131" s="157"/>
-      <c r="D131" s="157"/>
-      <c r="E131" s="157"/>
+      <c r="B131" s="156"/>
+      <c r="C131" s="156"/>
+      <c r="D131" s="156"/>
+      <c r="E131" s="156"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -4468,14 +4460,16 @@
         <f t="shared" si="3"/>
         <v>263677.82</v>
       </c>
-      <c r="L17" s="88"/>
+      <c r="L17" s="88">
+        <v>20000</v>
+      </c>
       <c r="M17" s="2">
         <f t="shared" si="4"/>
-        <v>286501.30734444817</v>
+        <v>306501.30734444817</v>
       </c>
       <c r="N17" s="5">
         <f t="shared" si="1"/>
-        <v>303691.38578511507</v>
+        <v>324891.38578511507</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
@@ -4514,7 +4508,7 @@
         <f t="shared" si="3"/>
         <v>218322.16</v>
       </c>
-      <c r="L18" s="153">
+      <c r="L18" s="88">
         <v>20000</v>
       </c>
       <c r="M18" s="2">
@@ -6038,15 +6032,15 @@
       </c>
       <c r="L52" s="87">
         <f>SUM(L7:L51)</f>
-        <v>20000</v>
+        <v>40000</v>
       </c>
       <c r="M52" s="22">
         <f>SUM(M7:M51)</f>
-        <v>6479211.0980660357</v>
+        <v>6499211.0980660357</v>
       </c>
       <c r="N52" s="21">
         <f>SUM(N7:N51)</f>
-        <v>6867963.7639499977</v>
+        <v>6889163.7639499977</v>
       </c>
       <c r="P52" s="50"/>
     </row>
@@ -6057,32 +6051,32 @@
       </c>
     </row>
     <row r="54" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="208"/>
-      <c r="D54" s="208"/>
-      <c r="E54" s="208"/>
-      <c r="F54" s="208"/>
-      <c r="G54" s="208"/>
-      <c r="H54" s="208"/>
-      <c r="I54" s="208"/>
-      <c r="J54" s="208"/>
-      <c r="K54" s="208"/>
-      <c r="L54" s="208"/>
-      <c r="M54" s="208"/>
-      <c r="N54" s="208"/>
+      <c r="C54" s="184"/>
+      <c r="D54" s="184"/>
+      <c r="E54" s="184"/>
+      <c r="F54" s="184"/>
+      <c r="G54" s="184"/>
+      <c r="H54" s="184"/>
+      <c r="I54" s="184"/>
+      <c r="J54" s="184"/>
+      <c r="K54" s="184"/>
+      <c r="L54" s="184"/>
+      <c r="M54" s="184"/>
+      <c r="N54" s="184"/>
     </row>
     <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="208"/>
-      <c r="D55" s="208"/>
-      <c r="E55" s="208"/>
-      <c r="F55" s="208"/>
-      <c r="G55" s="208"/>
-      <c r="H55" s="208"/>
-      <c r="I55" s="208"/>
-      <c r="J55" s="208"/>
-      <c r="K55" s="208"/>
-      <c r="L55" s="208"/>
-      <c r="M55" s="208"/>
-      <c r="N55" s="208"/>
+      <c r="C55" s="184"/>
+      <c r="D55" s="184"/>
+      <c r="E55" s="184"/>
+      <c r="F55" s="184"/>
+      <c r="G55" s="184"/>
+      <c r="H55" s="184"/>
+      <c r="I55" s="184"/>
+      <c r="J55" s="184"/>
+      <c r="K55" s="184"/>
+      <c r="L55" s="184"/>
+      <c r="M55" s="184"/>
+      <c r="N55" s="184"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C56" s="70"/>
@@ -6099,107 +6093,109 @@
       <c r="N56" s="70"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C57" s="208" t="s">
+      <c r="C57" s="184" t="s">
         <v>99</v>
       </c>
-      <c r="D57" s="208"/>
-      <c r="E57" s="208"/>
-      <c r="F57" s="208"/>
-      <c r="G57" s="208"/>
-      <c r="H57" s="208"/>
-      <c r="I57" s="208"/>
-      <c r="J57" s="208"/>
-      <c r="K57" s="208"/>
-      <c r="L57" s="208"/>
-      <c r="M57" s="208"/>
-      <c r="N57" s="208"/>
+      <c r="D57" s="184"/>
+      <c r="E57" s="184"/>
+      <c r="F57" s="184"/>
+      <c r="G57" s="184"/>
+      <c r="H57" s="184"/>
+      <c r="I57" s="184"/>
+      <c r="J57" s="184"/>
+      <c r="K57" s="184"/>
+      <c r="L57" s="184"/>
+      <c r="M57" s="184"/>
+      <c r="N57" s="184"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C58" s="208"/>
-      <c r="D58" s="208"/>
-      <c r="E58" s="208"/>
-      <c r="F58" s="208"/>
-      <c r="G58" s="208"/>
-      <c r="H58" s="208"/>
-      <c r="I58" s="208"/>
-      <c r="J58" s="208"/>
-      <c r="K58" s="208"/>
-      <c r="L58" s="208"/>
-      <c r="M58" s="208"/>
-      <c r="N58" s="208"/>
+      <c r="C58" s="184"/>
+      <c r="D58" s="184"/>
+      <c r="E58" s="184"/>
+      <c r="F58" s="184"/>
+      <c r="G58" s="184"/>
+      <c r="H58" s="184"/>
+      <c r="I58" s="184"/>
+      <c r="J58" s="184"/>
+      <c r="K58" s="184"/>
+      <c r="L58" s="184"/>
+      <c r="M58" s="184"/>
+      <c r="N58" s="184"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C59" s="208"/>
-      <c r="D59" s="208"/>
-      <c r="E59" s="208"/>
-      <c r="F59" s="208"/>
-      <c r="G59" s="208"/>
-      <c r="H59" s="208"/>
-      <c r="I59" s="208"/>
-      <c r="J59" s="208"/>
-      <c r="K59" s="208"/>
-      <c r="L59" s="208"/>
-      <c r="M59" s="208"/>
-      <c r="N59" s="208"/>
+      <c r="C59" s="184"/>
+      <c r="D59" s="184"/>
+      <c r="E59" s="184"/>
+      <c r="F59" s="184"/>
+      <c r="G59" s="184"/>
+      <c r="H59" s="184"/>
+      <c r="I59" s="184"/>
+      <c r="J59" s="184"/>
+      <c r="K59" s="184"/>
+      <c r="L59" s="184"/>
+      <c r="M59" s="184"/>
+      <c r="N59" s="184"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C60" s="208"/>
-      <c r="D60" s="208"/>
-      <c r="E60" s="208"/>
-      <c r="F60" s="208"/>
-      <c r="G60" s="208"/>
-      <c r="H60" s="208"/>
-      <c r="I60" s="208"/>
-      <c r="J60" s="208"/>
-      <c r="K60" s="208"/>
-      <c r="L60" s="208"/>
-      <c r="M60" s="208"/>
-      <c r="N60" s="208"/>
+      <c r="C60" s="184"/>
+      <c r="D60" s="184"/>
+      <c r="E60" s="184"/>
+      <c r="F60" s="184"/>
+      <c r="G60" s="184"/>
+      <c r="H60" s="184"/>
+      <c r="I60" s="184"/>
+      <c r="J60" s="184"/>
+      <c r="K60" s="184"/>
+      <c r="L60" s="184"/>
+      <c r="M60" s="184"/>
+      <c r="N60" s="184"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C61" s="208"/>
-      <c r="D61" s="208"/>
-      <c r="E61" s="208"/>
-      <c r="F61" s="208"/>
-      <c r="G61" s="208"/>
-      <c r="H61" s="208"/>
-      <c r="I61" s="208"/>
-      <c r="J61" s="208"/>
-      <c r="K61" s="208"/>
-      <c r="L61" s="208"/>
-      <c r="M61" s="208"/>
-      <c r="N61" s="208"/>
+      <c r="C61" s="184"/>
+      <c r="D61" s="184"/>
+      <c r="E61" s="184"/>
+      <c r="F61" s="184"/>
+      <c r="G61" s="184"/>
+      <c r="H61" s="184"/>
+      <c r="I61" s="184"/>
+      <c r="J61" s="184"/>
+      <c r="K61" s="184"/>
+      <c r="L61" s="184"/>
+      <c r="M61" s="184"/>
+      <c r="N61" s="184"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C62" s="208"/>
-      <c r="D62" s="208"/>
-      <c r="E62" s="208"/>
-      <c r="F62" s="208"/>
-      <c r="G62" s="208"/>
-      <c r="H62" s="208"/>
-      <c r="I62" s="208"/>
-      <c r="J62" s="208"/>
-      <c r="K62" s="208"/>
-      <c r="L62" s="208"/>
-      <c r="M62" s="208"/>
-      <c r="N62" s="208"/>
+      <c r="C62" s="184"/>
+      <c r="D62" s="184"/>
+      <c r="E62" s="184"/>
+      <c r="F62" s="184"/>
+      <c r="G62" s="184"/>
+      <c r="H62" s="184"/>
+      <c r="I62" s="184"/>
+      <c r="J62" s="184"/>
+      <c r="K62" s="184"/>
+      <c r="L62" s="184"/>
+      <c r="M62" s="184"/>
+      <c r="N62" s="184"/>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C63" s="208"/>
-      <c r="D63" s="208"/>
-      <c r="E63" s="208"/>
-      <c r="F63" s="208"/>
-      <c r="G63" s="208"/>
-      <c r="H63" s="208"/>
-      <c r="I63" s="208"/>
-      <c r="J63" s="208"/>
-      <c r="K63" s="208"/>
-      <c r="L63" s="208"/>
-      <c r="M63" s="208"/>
-      <c r="N63" s="208"/>
+      <c r="C63" s="184"/>
+      <c r="D63" s="184"/>
+      <c r="E63" s="184"/>
+      <c r="F63" s="184"/>
+      <c r="G63" s="184"/>
+      <c r="H63" s="184"/>
+      <c r="I63" s="184"/>
+      <c r="J63" s="184"/>
+      <c r="K63" s="184"/>
+      <c r="L63" s="184"/>
+      <c r="M63" s="184"/>
+      <c r="N63" s="184"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
     <mergeCell ref="C57:N63"/>
     <mergeCell ref="C54:N55"/>
     <mergeCell ref="L1:M1"/>
@@ -6216,8 +6212,6 @@
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:C6"/>
     <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="3" orientation="landscape" r:id="rId1"/>

</xml_diff>